<commit_message>
vault backup: 2026-07-18 12:18:41
</commit_message>
<xml_diff>
--- a/resources/workout/Fauzan_Training_Log.xlsx
+++ b/resources/workout/Fauzan_Training_Log.xlsx
@@ -465,10 +465,10 @@
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="165" xfId="0" applyNumberFormat="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
     </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
     </xf>
@@ -1794,20 +1794,19 @@
     </row>
     <row r="5">
       <c r="A5" s="6"/>
-      <c r="B5" s="8"/>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="8" t="s">
         <v>89</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="E5" s="8">
+      <c r="E5" s="9">
         <v>2</v>
       </c>
       <c r="F5" s="7">
         <v>12</v>
       </c>
-      <c r="G5" s="8">
+      <c r="G5" s="9">
         <v>25</v>
       </c>
       <c r="H5" s="7"/>
@@ -1820,7 +1819,7 @@
         <v>300</v>
       </c>
       <c r="M5" s="7"/>
-      <c r="N5" s="8" t="s">
+      <c r="N5" s="9" t="s">
         <v>88</v>
       </c>
       <c r="O5" s="5" t="s">
@@ -1829,10 +1828,6 @@
     </row>
     <row r="6">
       <c r="A6" s="6"/>
-      <c r="B6" t="str">
-        <f t="shared" ref="B6:B9" si="0">IF(A6="","",WEEKNUM(A6,2))</f>
-        <v/>
-      </c>
       <c r="C6" t="s">
         <v>46</v>
       </c>
@@ -1858,17 +1853,13 @@
         <v>120</v>
       </c>
       <c r="M6" s="7"/>
-      <c r="N6" s="8" t="s">
+      <c r="N6" s="9" t="s">
         <v>88</v>
       </c>
       <c r="O6" s="3"/>
     </row>
     <row r="7">
       <c r="A7" s="6"/>
-      <c r="B7" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
       <c r="C7" t="s">
         <v>89</v>
       </c>
@@ -1892,17 +1883,13 @@
         <v/>
       </c>
       <c r="M7" s="7"/>
-      <c r="N7" s="8" t="s">
+      <c r="N7" s="9" t="s">
         <v>88</v>
       </c>
       <c r="O7" s="3"/>
     </row>
     <row r="8">
       <c r="A8" s="6"/>
-      <c r="B8" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
       <c r="C8" s="10" t="s">
         <v>46</v>
       </c>
@@ -1926,17 +1913,13 @@
         <v/>
       </c>
       <c r="M8" s="7"/>
-      <c r="N8" s="8" t="s">
+      <c r="N8" s="9" t="s">
         <v>88</v>
       </c>
       <c r="O8" s="3"/>
     </row>
     <row r="9">
       <c r="A9" s="6"/>
-      <c r="B9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
       <c r="C9" t="s">
         <v>46</v>
       </c>
@@ -1960,7 +1943,7 @@
         <v/>
       </c>
       <c r="M9" s="7"/>
-      <c r="N9" s="8" t="s">
+      <c r="N9" s="9" t="s">
         <v>88</v>
       </c>
       <c r="O9" s="5" t="s">
@@ -1969,10 +1952,6 @@
     </row>
     <row r="10">
       <c r="A10" s="6"/>
-      <c r="B10" t="str">
-        <f t="shared" ref="B10:B73" si="1">IF(A10="","",WEEKNUM(A10,2))</f>
-        <v/>
-      </c>
       <c r="C10" s="10" t="s">
         <v>46</v>
       </c>
@@ -1994,21 +1973,17 @@
         <v>8</v>
       </c>
       <c r="L10" s="7">
-        <f t="shared" ref="L10:L73" si="2">IF(OR(F10="",G10=""),"",F10*G10)</f>
+        <f t="shared" ref="L10:L73" si="0">IF(OR(F10="",G10=""),"",F10*G10)</f>
         <v>180</v>
       </c>
       <c r="M10" s="7"/>
-      <c r="N10" s="8" t="s">
+      <c r="N10" s="9" t="s">
         <v>88</v>
       </c>
       <c r="O10" s="3"/>
     </row>
     <row r="11">
       <c r="A11" s="6"/>
-      <c r="B11" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
       <c r="C11" t="s">
         <v>46</v>
       </c>
@@ -2028,7 +2003,7 @@
         <v>7</v>
       </c>
       <c r="L11" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M11" s="7"/>
@@ -2039,16 +2014,12 @@
     </row>
     <row r="12">
       <c r="A12" s="6"/>
-      <c r="B12" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
       <c r="F12" s="7"/>
       <c r="H12" s="7"/>
       <c r="I12" s="7"/>
       <c r="K12" s="7"/>
       <c r="L12" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M12" s="7"/>
@@ -2057,7 +2028,7 @@
     <row r="13">
       <c r="A13" s="6"/>
       <c r="B13" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="B13:B76" si="1">IF(A13="","",WEEKNUM(A13,2))</f>
         <v/>
       </c>
       <c r="F13" s="7"/>
@@ -2065,7 +2036,7 @@
       <c r="I13" s="7"/>
       <c r="K13" s="7"/>
       <c r="L13" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M13" s="7"/>
@@ -2082,7 +2053,7 @@
       <c r="I14" s="7"/>
       <c r="K14" s="7"/>
       <c r="L14" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M14" s="7"/>
@@ -2099,7 +2070,7 @@
       <c r="I15" s="7"/>
       <c r="K15" s="7"/>
       <c r="L15" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M15" s="7"/>
@@ -2116,7 +2087,7 @@
       <c r="I16" s="7"/>
       <c r="K16" s="7"/>
       <c r="L16" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M16" s="7"/>
@@ -2133,7 +2104,7 @@
       <c r="I17" s="7"/>
       <c r="K17" s="7"/>
       <c r="L17" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M17" s="7"/>
@@ -2150,7 +2121,7 @@
       <c r="I18" s="7"/>
       <c r="K18" s="7"/>
       <c r="L18" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M18" s="7"/>
@@ -2167,7 +2138,7 @@
       <c r="I19" s="7"/>
       <c r="K19" s="7"/>
       <c r="L19" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M19" s="7"/>
@@ -2184,7 +2155,7 @@
       <c r="I20" s="7"/>
       <c r="K20" s="7"/>
       <c r="L20" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M20" s="7"/>
@@ -2201,7 +2172,7 @@
       <c r="I21" s="7"/>
       <c r="K21" s="7"/>
       <c r="L21" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M21" s="7"/>
@@ -2218,7 +2189,7 @@
       <c r="I22" s="7"/>
       <c r="K22" s="7"/>
       <c r="L22" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M22" s="7"/>
@@ -2235,7 +2206,7 @@
       <c r="I23" s="7"/>
       <c r="K23" s="7"/>
       <c r="L23" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M23" s="7"/>
@@ -2252,7 +2223,7 @@
       <c r="I24" s="7"/>
       <c r="K24" s="7"/>
       <c r="L24" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M24" s="7"/>
@@ -2269,7 +2240,7 @@
       <c r="I25" s="7"/>
       <c r="K25" s="7"/>
       <c r="L25" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M25" s="7"/>
@@ -2286,7 +2257,7 @@
       <c r="I26" s="7"/>
       <c r="K26" s="7"/>
       <c r="L26" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M26" s="7"/>
@@ -2303,7 +2274,7 @@
       <c r="I27" s="7"/>
       <c r="K27" s="7"/>
       <c r="L27" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M27" s="7"/>
@@ -2320,7 +2291,7 @@
       <c r="I28" s="7"/>
       <c r="K28" s="7"/>
       <c r="L28" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M28" s="7"/>
@@ -2337,7 +2308,7 @@
       <c r="I29" s="7"/>
       <c r="K29" s="7"/>
       <c r="L29" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M29" s="7"/>
@@ -2354,7 +2325,7 @@
       <c r="I30" s="7"/>
       <c r="K30" s="7"/>
       <c r="L30" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M30" s="7"/>
@@ -2371,7 +2342,7 @@
       <c r="I31" s="7"/>
       <c r="K31" s="7"/>
       <c r="L31" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M31" s="7"/>
@@ -2388,7 +2359,7 @@
       <c r="I32" s="7"/>
       <c r="K32" s="7"/>
       <c r="L32" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M32" s="7"/>
@@ -2405,7 +2376,7 @@
       <c r="I33" s="7"/>
       <c r="K33" s="7"/>
       <c r="L33" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M33" s="7"/>
@@ -2422,7 +2393,7 @@
       <c r="I34" s="7"/>
       <c r="K34" s="7"/>
       <c r="L34" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M34" s="7"/>
@@ -2439,7 +2410,7 @@
       <c r="I35" s="7"/>
       <c r="K35" s="7"/>
       <c r="L35" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M35" s="7"/>
@@ -2456,7 +2427,7 @@
       <c r="I36" s="7"/>
       <c r="K36" s="7"/>
       <c r="L36" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M36" s="7"/>
@@ -2473,7 +2444,7 @@
       <c r="I37" s="7"/>
       <c r="K37" s="7"/>
       <c r="L37" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M37" s="7"/>
@@ -2490,7 +2461,7 @@
       <c r="I38" s="7"/>
       <c r="K38" s="7"/>
       <c r="L38" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M38" s="7"/>
@@ -2507,7 +2478,7 @@
       <c r="I39" s="7"/>
       <c r="K39" s="7"/>
       <c r="L39" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M39" s="7"/>
@@ -2524,7 +2495,7 @@
       <c r="I40" s="7"/>
       <c r="K40" s="7"/>
       <c r="L40" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M40" s="7"/>
@@ -2541,7 +2512,7 @@
       <c r="I41" s="7"/>
       <c r="K41" s="7"/>
       <c r="L41" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M41" s="7"/>
@@ -2558,7 +2529,7 @@
       <c r="I42" s="7"/>
       <c r="K42" s="7"/>
       <c r="L42" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M42" s="7"/>
@@ -2575,7 +2546,7 @@
       <c r="I43" s="7"/>
       <c r="K43" s="7"/>
       <c r="L43" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M43" s="7"/>
@@ -2592,7 +2563,7 @@
       <c r="I44" s="7"/>
       <c r="K44" s="7"/>
       <c r="L44" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M44" s="7"/>
@@ -2609,7 +2580,7 @@
       <c r="I45" s="7"/>
       <c r="K45" s="7"/>
       <c r="L45" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M45" s="7"/>
@@ -2626,7 +2597,7 @@
       <c r="I46" s="7"/>
       <c r="K46" s="7"/>
       <c r="L46" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M46" s="7"/>
@@ -2643,7 +2614,7 @@
       <c r="I47" s="7"/>
       <c r="K47" s="7"/>
       <c r="L47" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M47" s="7"/>
@@ -2660,7 +2631,7 @@
       <c r="I48" s="7"/>
       <c r="K48" s="7"/>
       <c r="L48" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M48" s="7"/>
@@ -2677,7 +2648,7 @@
       <c r="I49" s="7"/>
       <c r="K49" s="7"/>
       <c r="L49" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M49" s="7"/>
@@ -2694,7 +2665,7 @@
       <c r="I50" s="7"/>
       <c r="K50" s="7"/>
       <c r="L50" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M50" s="7"/>
@@ -2711,7 +2682,7 @@
       <c r="I51" s="7"/>
       <c r="K51" s="7"/>
       <c r="L51" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M51" s="7"/>
@@ -2728,7 +2699,7 @@
       <c r="I52" s="7"/>
       <c r="K52" s="7"/>
       <c r="L52" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M52" s="7"/>
@@ -2745,7 +2716,7 @@
       <c r="I53" s="7"/>
       <c r="K53" s="7"/>
       <c r="L53" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M53" s="7"/>
@@ -2762,7 +2733,7 @@
       <c r="I54" s="7"/>
       <c r="K54" s="7"/>
       <c r="L54" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M54" s="7"/>
@@ -2779,7 +2750,7 @@
       <c r="I55" s="7"/>
       <c r="K55" s="7"/>
       <c r="L55" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M55" s="7"/>
@@ -2796,7 +2767,7 @@
       <c r="I56" s="7"/>
       <c r="K56" s="7"/>
       <c r="L56" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M56" s="7"/>
@@ -2813,7 +2784,7 @@
       <c r="I57" s="7"/>
       <c r="K57" s="7"/>
       <c r="L57" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M57" s="7"/>
@@ -2830,7 +2801,7 @@
       <c r="I58" s="7"/>
       <c r="K58" s="7"/>
       <c r="L58" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M58" s="7"/>
@@ -2847,7 +2818,7 @@
       <c r="I59" s="7"/>
       <c r="K59" s="7"/>
       <c r="L59" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M59" s="7"/>
@@ -2864,7 +2835,7 @@
       <c r="I60" s="7"/>
       <c r="K60" s="7"/>
       <c r="L60" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M60" s="7"/>
@@ -2881,7 +2852,7 @@
       <c r="I61" s="7"/>
       <c r="K61" s="7"/>
       <c r="L61" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M61" s="7"/>
@@ -2898,7 +2869,7 @@
       <c r="I62" s="7"/>
       <c r="K62" s="7"/>
       <c r="L62" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M62" s="7"/>
@@ -2915,7 +2886,7 @@
       <c r="I63" s="7"/>
       <c r="K63" s="7"/>
       <c r="L63" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M63" s="7"/>
@@ -2932,7 +2903,7 @@
       <c r="I64" s="7"/>
       <c r="K64" s="7"/>
       <c r="L64" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M64" s="7"/>
@@ -2949,7 +2920,7 @@
       <c r="I65" s="7"/>
       <c r="K65" s="7"/>
       <c r="L65" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M65" s="7"/>
@@ -2966,7 +2937,7 @@
       <c r="I66" s="7"/>
       <c r="K66" s="7"/>
       <c r="L66" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M66" s="7"/>
@@ -2983,7 +2954,7 @@
       <c r="I67" s="7"/>
       <c r="K67" s="7"/>
       <c r="L67" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M67" s="7"/>
@@ -3000,7 +2971,7 @@
       <c r="I68" s="7"/>
       <c r="K68" s="7"/>
       <c r="L68" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M68" s="7"/>
@@ -3017,7 +2988,7 @@
       <c r="I69" s="7"/>
       <c r="K69" s="7"/>
       <c r="L69" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M69" s="7"/>
@@ -3034,7 +3005,7 @@
       <c r="I70" s="7"/>
       <c r="K70" s="7"/>
       <c r="L70" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M70" s="7"/>
@@ -3051,7 +3022,7 @@
       <c r="I71" s="7"/>
       <c r="K71" s="7"/>
       <c r="L71" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M71" s="7"/>
@@ -3068,7 +3039,7 @@
       <c r="I72" s="7"/>
       <c r="K72" s="7"/>
       <c r="L72" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M72" s="7"/>
@@ -3085,7 +3056,7 @@
       <c r="I73" s="7"/>
       <c r="K73" s="7"/>
       <c r="L73" s="7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="M73" s="7"/>
@@ -3094,7 +3065,7 @@
     <row r="74">
       <c r="A74" s="6"/>
       <c r="B74" t="str">
-        <f t="shared" ref="B74:B99" si="3">IF(A74="","",WEEKNUM(A74,2))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="F74" s="7"/>
@@ -3102,7 +3073,7 @@
       <c r="I74" s="7"/>
       <c r="K74" s="7"/>
       <c r="L74" s="7" t="str">
-        <f t="shared" ref="L74:L99" si="4">IF(OR(F74="",G74=""),"",F74*G74)</f>
+        <f t="shared" ref="L74:L99" si="2">IF(OR(F74="",G74=""),"",F74*G74)</f>
         <v/>
       </c>
       <c r="M74" s="7"/>
@@ -3111,7 +3082,7 @@
     <row r="75">
       <c r="A75" s="6"/>
       <c r="B75" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="F75" s="7"/>
@@ -3119,7 +3090,7 @@
       <c r="I75" s="7"/>
       <c r="K75" s="7"/>
       <c r="L75" s="7" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="M75" s="7"/>
@@ -3128,7 +3099,7 @@
     <row r="76">
       <c r="A76" s="6"/>
       <c r="B76" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="F76" s="7"/>
@@ -3136,7 +3107,7 @@
       <c r="I76" s="7"/>
       <c r="K76" s="7"/>
       <c r="L76" s="7" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="M76" s="7"/>
@@ -3145,7 +3116,7 @@
     <row r="77">
       <c r="A77" s="6"/>
       <c r="B77" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="B77:B99" si="3">IF(A77="","",WEEKNUM(A77,2))</f>
         <v/>
       </c>
       <c r="F77" s="7"/>
@@ -3153,7 +3124,7 @@
       <c r="I77" s="7"/>
       <c r="K77" s="7"/>
       <c r="L77" s="7" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="M77" s="7"/>
@@ -3170,7 +3141,7 @@
       <c r="I78" s="7"/>
       <c r="K78" s="7"/>
       <c r="L78" s="7" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="M78" s="7"/>
@@ -3187,7 +3158,7 @@
       <c r="I79" s="7"/>
       <c r="K79" s="7"/>
       <c r="L79" s="7" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="M79" s="7"/>
@@ -3204,7 +3175,7 @@
       <c r="I80" s="7"/>
       <c r="K80" s="7"/>
       <c r="L80" s="7" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="M80" s="7"/>
@@ -3221,7 +3192,7 @@
       <c r="I81" s="7"/>
       <c r="K81" s="7"/>
       <c r="L81" s="7" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="M81" s="7"/>
@@ -3238,7 +3209,7 @@
       <c r="I82" s="7"/>
       <c r="K82" s="7"/>
       <c r="L82" s="7" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="M82" s="7"/>
@@ -3255,7 +3226,7 @@
       <c r="I83" s="7"/>
       <c r="K83" s="7"/>
       <c r="L83" s="7" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="M83" s="7"/>
@@ -3272,7 +3243,7 @@
       <c r="I84" s="7"/>
       <c r="K84" s="7"/>
       <c r="L84" s="7" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="M84" s="7"/>
@@ -3289,7 +3260,7 @@
       <c r="I85" s="7"/>
       <c r="K85" s="7"/>
       <c r="L85" s="7" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="M85" s="7"/>
@@ -3306,7 +3277,7 @@
       <c r="I86" s="7"/>
       <c r="K86" s="7"/>
       <c r="L86" s="7" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="M86" s="7"/>
@@ -3323,7 +3294,7 @@
       <c r="I87" s="7"/>
       <c r="K87" s="7"/>
       <c r="L87" s="7" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="M87" s="7"/>
@@ -3340,7 +3311,7 @@
       <c r="I88" s="7"/>
       <c r="K88" s="7"/>
       <c r="L88" s="7" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="M88" s="7"/>
@@ -3357,7 +3328,7 @@
       <c r="I89" s="7"/>
       <c r="K89" s="7"/>
       <c r="L89" s="7" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="M89" s="7"/>
@@ -3374,7 +3345,7 @@
       <c r="I90" s="7"/>
       <c r="K90" s="7"/>
       <c r="L90" s="7" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="M90" s="7"/>
@@ -3391,7 +3362,7 @@
       <c r="I91" s="7"/>
       <c r="K91" s="7"/>
       <c r="L91" s="7" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="M91" s="7"/>
@@ -3408,7 +3379,7 @@
       <c r="I92" s="7"/>
       <c r="K92" s="7"/>
       <c r="L92" s="7" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="M92" s="7"/>
@@ -3425,7 +3396,7 @@
       <c r="I93" s="7"/>
       <c r="K93" s="7"/>
       <c r="L93" s="7" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="M93" s="7"/>
@@ -3442,7 +3413,7 @@
       <c r="I94" s="7"/>
       <c r="K94" s="7"/>
       <c r="L94" s="7" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="M94" s="7"/>
@@ -3459,7 +3430,7 @@
       <c r="I95" s="7"/>
       <c r="K95" s="7"/>
       <c r="L95" s="7" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="M95" s="7"/>
@@ -3476,7 +3447,7 @@
       <c r="I96" s="7"/>
       <c r="K96" s="7"/>
       <c r="L96" s="7" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="M96" s="7"/>
@@ -3493,7 +3464,7 @@
       <c r="I97" s="7"/>
       <c r="K97" s="7"/>
       <c r="L97" s="7" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="M97" s="7"/>
@@ -3510,7 +3481,7 @@
       <c r="I98" s="7"/>
       <c r="K98" s="7"/>
       <c r="L98" s="7" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="M98" s="7"/>
@@ -3527,7 +3498,7 @@
       <c r="I99" s="7"/>
       <c r="K99" s="7"/>
       <c r="L99" s="7" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="M99" s="7"/>
@@ -3536,7 +3507,7 @@
     <row r="100">
       <c r="A100" s="6"/>
       <c r="B100" t="str">
-        <f t="shared" ref="B100:B163" si="5">IF(A100="","",WEEKNUM(A100,2))</f>
+        <f t="shared" ref="B100:B163" si="4">IF(A100="","",WEEKNUM(A100,2))</f>
         <v/>
       </c>
       <c r="F100" s="7"/>
@@ -3544,7 +3515,7 @@
       <c r="I100" s="7"/>
       <c r="K100" s="7"/>
       <c r="L100" s="7" t="str">
-        <f t="shared" ref="L100:L163" si="6">IF(OR(F100="",G100=""),"",F100*G100)</f>
+        <f t="shared" ref="L100:L163" si="5">IF(OR(F100="",G100=""),"",F100*G100)</f>
         <v/>
       </c>
       <c r="M100" s="7"/>
@@ -3553,7 +3524,7 @@
     <row r="101">
       <c r="A101" s="6"/>
       <c r="B101" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F101" s="7"/>
@@ -3561,7 +3532,7 @@
       <c r="I101" s="7"/>
       <c r="K101" s="7"/>
       <c r="L101" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M101" s="7"/>
@@ -3570,7 +3541,7 @@
     <row r="102">
       <c r="A102" s="6"/>
       <c r="B102" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F102" s="7"/>
@@ -3578,7 +3549,7 @@
       <c r="I102" s="7"/>
       <c r="K102" s="7"/>
       <c r="L102" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M102" s="7"/>
@@ -3587,7 +3558,7 @@
     <row r="103">
       <c r="A103" s="6"/>
       <c r="B103" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F103" s="7"/>
@@ -3595,7 +3566,7 @@
       <c r="I103" s="7"/>
       <c r="K103" s="7"/>
       <c r="L103" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M103" s="7"/>
@@ -3604,7 +3575,7 @@
     <row r="104">
       <c r="A104" s="6"/>
       <c r="B104" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F104" s="7"/>
@@ -3612,7 +3583,7 @@
       <c r="I104" s="7"/>
       <c r="K104" s="7"/>
       <c r="L104" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M104" s="7"/>
@@ -3621,7 +3592,7 @@
     <row r="105">
       <c r="A105" s="6"/>
       <c r="B105" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F105" s="7"/>
@@ -3629,7 +3600,7 @@
       <c r="I105" s="7"/>
       <c r="K105" s="7"/>
       <c r="L105" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M105" s="7"/>
@@ -3638,7 +3609,7 @@
     <row r="106">
       <c r="A106" s="6"/>
       <c r="B106" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F106" s="7"/>
@@ -3646,7 +3617,7 @@
       <c r="I106" s="7"/>
       <c r="K106" s="7"/>
       <c r="L106" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M106" s="7"/>
@@ -3655,7 +3626,7 @@
     <row r="107">
       <c r="A107" s="6"/>
       <c r="B107" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F107" s="7"/>
@@ -3663,7 +3634,7 @@
       <c r="I107" s="7"/>
       <c r="K107" s="7"/>
       <c r="L107" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M107" s="7"/>
@@ -3672,7 +3643,7 @@
     <row r="108">
       <c r="A108" s="6"/>
       <c r="B108" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F108" s="7"/>
@@ -3680,7 +3651,7 @@
       <c r="I108" s="7"/>
       <c r="K108" s="7"/>
       <c r="L108" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M108" s="7"/>
@@ -3689,7 +3660,7 @@
     <row r="109">
       <c r="A109" s="6"/>
       <c r="B109" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F109" s="7"/>
@@ -3697,7 +3668,7 @@
       <c r="I109" s="7"/>
       <c r="K109" s="7"/>
       <c r="L109" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M109" s="7"/>
@@ -3706,7 +3677,7 @@
     <row r="110">
       <c r="A110" s="6"/>
       <c r="B110" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F110" s="7"/>
@@ -3714,7 +3685,7 @@
       <c r="I110" s="7"/>
       <c r="K110" s="7"/>
       <c r="L110" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M110" s="7"/>
@@ -3723,7 +3694,7 @@
     <row r="111">
       <c r="A111" s="6"/>
       <c r="B111" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F111" s="7"/>
@@ -3731,7 +3702,7 @@
       <c r="I111" s="7"/>
       <c r="K111" s="7"/>
       <c r="L111" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M111" s="7"/>
@@ -3740,7 +3711,7 @@
     <row r="112">
       <c r="A112" s="6"/>
       <c r="B112" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F112" s="7"/>
@@ -3748,7 +3719,7 @@
       <c r="I112" s="7"/>
       <c r="K112" s="7"/>
       <c r="L112" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M112" s="7"/>
@@ -3757,7 +3728,7 @@
     <row r="113">
       <c r="A113" s="6"/>
       <c r="B113" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F113" s="7"/>
@@ -3765,7 +3736,7 @@
       <c r="I113" s="7"/>
       <c r="K113" s="7"/>
       <c r="L113" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M113" s="7"/>
@@ -3774,7 +3745,7 @@
     <row r="114">
       <c r="A114" s="6"/>
       <c r="B114" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F114" s="7"/>
@@ -3782,7 +3753,7 @@
       <c r="I114" s="7"/>
       <c r="K114" s="7"/>
       <c r="L114" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M114" s="7"/>
@@ -3791,7 +3762,7 @@
     <row r="115">
       <c r="A115" s="6"/>
       <c r="B115" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F115" s="7"/>
@@ -3799,7 +3770,7 @@
       <c r="I115" s="7"/>
       <c r="K115" s="7"/>
       <c r="L115" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M115" s="7"/>
@@ -3808,7 +3779,7 @@
     <row r="116">
       <c r="A116" s="6"/>
       <c r="B116" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F116" s="7"/>
@@ -3816,7 +3787,7 @@
       <c r="I116" s="7"/>
       <c r="K116" s="7"/>
       <c r="L116" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M116" s="7"/>
@@ -3825,7 +3796,7 @@
     <row r="117">
       <c r="A117" s="6"/>
       <c r="B117" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F117" s="7"/>
@@ -3833,7 +3804,7 @@
       <c r="I117" s="7"/>
       <c r="K117" s="7"/>
       <c r="L117" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M117" s="7"/>
@@ -3842,7 +3813,7 @@
     <row r="118">
       <c r="A118" s="6"/>
       <c r="B118" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F118" s="7"/>
@@ -3850,7 +3821,7 @@
       <c r="I118" s="7"/>
       <c r="K118" s="7"/>
       <c r="L118" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M118" s="7"/>
@@ -3859,7 +3830,7 @@
     <row r="119">
       <c r="A119" s="6"/>
       <c r="B119" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F119" s="7"/>
@@ -3867,7 +3838,7 @@
       <c r="I119" s="7"/>
       <c r="K119" s="7"/>
       <c r="L119" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M119" s="7"/>
@@ -3876,7 +3847,7 @@
     <row r="120">
       <c r="A120" s="6"/>
       <c r="B120" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F120" s="7"/>
@@ -3884,7 +3855,7 @@
       <c r="I120" s="7"/>
       <c r="K120" s="7"/>
       <c r="L120" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M120" s="7"/>
@@ -3893,7 +3864,7 @@
     <row r="121">
       <c r="A121" s="6"/>
       <c r="B121" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F121" s="7"/>
@@ -3901,7 +3872,7 @@
       <c r="I121" s="7"/>
       <c r="K121" s="7"/>
       <c r="L121" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M121" s="7"/>
@@ -3910,7 +3881,7 @@
     <row r="122">
       <c r="A122" s="6"/>
       <c r="B122" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F122" s="7"/>
@@ -3918,7 +3889,7 @@
       <c r="I122" s="7"/>
       <c r="K122" s="7"/>
       <c r="L122" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M122" s="7"/>
@@ -3927,7 +3898,7 @@
     <row r="123">
       <c r="A123" s="6"/>
       <c r="B123" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F123" s="7"/>
@@ -3935,7 +3906,7 @@
       <c r="I123" s="7"/>
       <c r="K123" s="7"/>
       <c r="L123" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M123" s="7"/>
@@ -3944,7 +3915,7 @@
     <row r="124">
       <c r="A124" s="6"/>
       <c r="B124" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F124" s="7"/>
@@ -3952,7 +3923,7 @@
       <c r="I124" s="7"/>
       <c r="K124" s="7"/>
       <c r="L124" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M124" s="7"/>
@@ -3961,7 +3932,7 @@
     <row r="125">
       <c r="A125" s="6"/>
       <c r="B125" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F125" s="7"/>
@@ -3969,7 +3940,7 @@
       <c r="I125" s="7"/>
       <c r="K125" s="7"/>
       <c r="L125" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M125" s="7"/>
@@ -3978,7 +3949,7 @@
     <row r="126">
       <c r="A126" s="6"/>
       <c r="B126" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F126" s="7"/>
@@ -3986,7 +3957,7 @@
       <c r="I126" s="7"/>
       <c r="K126" s="7"/>
       <c r="L126" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M126" s="7"/>
@@ -3995,7 +3966,7 @@
     <row r="127">
       <c r="A127" s="6"/>
       <c r="B127" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F127" s="7"/>
@@ -4003,7 +3974,7 @@
       <c r="I127" s="7"/>
       <c r="K127" s="7"/>
       <c r="L127" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M127" s="7"/>
@@ -4012,7 +3983,7 @@
     <row r="128">
       <c r="A128" s="6"/>
       <c r="B128" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F128" s="7"/>
@@ -4020,7 +3991,7 @@
       <c r="I128" s="7"/>
       <c r="K128" s="7"/>
       <c r="L128" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M128" s="7"/>
@@ -4029,7 +4000,7 @@
     <row r="129">
       <c r="A129" s="6"/>
       <c r="B129" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F129" s="7"/>
@@ -4037,7 +4008,7 @@
       <c r="I129" s="7"/>
       <c r="K129" s="7"/>
       <c r="L129" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M129" s="7"/>
@@ -4046,7 +4017,7 @@
     <row r="130">
       <c r="A130" s="6"/>
       <c r="B130" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F130" s="7"/>
@@ -4054,7 +4025,7 @@
       <c r="I130" s="7"/>
       <c r="K130" s="7"/>
       <c r="L130" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M130" s="7"/>
@@ -4063,7 +4034,7 @@
     <row r="131">
       <c r="A131" s="6"/>
       <c r="B131" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F131" s="7"/>
@@ -4071,7 +4042,7 @@
       <c r="I131" s="7"/>
       <c r="K131" s="7"/>
       <c r="L131" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M131" s="7"/>
@@ -4080,7 +4051,7 @@
     <row r="132">
       <c r="A132" s="6"/>
       <c r="B132" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F132" s="7"/>
@@ -4088,7 +4059,7 @@
       <c r="I132" s="7"/>
       <c r="K132" s="7"/>
       <c r="L132" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M132" s="7"/>
@@ -4097,7 +4068,7 @@
     <row r="133">
       <c r="A133" s="6"/>
       <c r="B133" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F133" s="7"/>
@@ -4105,7 +4076,7 @@
       <c r="I133" s="7"/>
       <c r="K133" s="7"/>
       <c r="L133" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M133" s="7"/>
@@ -4114,7 +4085,7 @@
     <row r="134">
       <c r="A134" s="6"/>
       <c r="B134" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F134" s="7"/>
@@ -4122,7 +4093,7 @@
       <c r="I134" s="7"/>
       <c r="K134" s="7"/>
       <c r="L134" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M134" s="7"/>
@@ -4131,7 +4102,7 @@
     <row r="135">
       <c r="A135" s="6"/>
       <c r="B135" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F135" s="7"/>
@@ -4139,7 +4110,7 @@
       <c r="I135" s="7"/>
       <c r="K135" s="7"/>
       <c r="L135" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M135" s="7"/>
@@ -4148,7 +4119,7 @@
     <row r="136">
       <c r="A136" s="6"/>
       <c r="B136" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F136" s="7"/>
@@ -4156,7 +4127,7 @@
       <c r="I136" s="7"/>
       <c r="K136" s="7"/>
       <c r="L136" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M136" s="7"/>
@@ -4165,7 +4136,7 @@
     <row r="137">
       <c r="A137" s="6"/>
       <c r="B137" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F137" s="7"/>
@@ -4173,7 +4144,7 @@
       <c r="I137" s="7"/>
       <c r="K137" s="7"/>
       <c r="L137" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M137" s="7"/>
@@ -4182,7 +4153,7 @@
     <row r="138">
       <c r="A138" s="6"/>
       <c r="B138" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F138" s="7"/>
@@ -4190,7 +4161,7 @@
       <c r="I138" s="7"/>
       <c r="K138" s="7"/>
       <c r="L138" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M138" s="7"/>
@@ -4199,7 +4170,7 @@
     <row r="139">
       <c r="A139" s="6"/>
       <c r="B139" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F139" s="7"/>
@@ -4207,7 +4178,7 @@
       <c r="I139" s="7"/>
       <c r="K139" s="7"/>
       <c r="L139" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M139" s="7"/>
@@ -4216,7 +4187,7 @@
     <row r="140">
       <c r="A140" s="6"/>
       <c r="B140" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F140" s="7"/>
@@ -4224,7 +4195,7 @@
       <c r="I140" s="7"/>
       <c r="K140" s="7"/>
       <c r="L140" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M140" s="7"/>
@@ -4233,7 +4204,7 @@
     <row r="141">
       <c r="A141" s="6"/>
       <c r="B141" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F141" s="7"/>
@@ -4241,7 +4212,7 @@
       <c r="I141" s="7"/>
       <c r="K141" s="7"/>
       <c r="L141" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M141" s="7"/>
@@ -4250,7 +4221,7 @@
     <row r="142">
       <c r="A142" s="6"/>
       <c r="B142" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F142" s="7"/>
@@ -4258,7 +4229,7 @@
       <c r="I142" s="7"/>
       <c r="K142" s="7"/>
       <c r="L142" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M142" s="7"/>
@@ -4267,7 +4238,7 @@
     <row r="143">
       <c r="A143" s="6"/>
       <c r="B143" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F143" s="7"/>
@@ -4275,7 +4246,7 @@
       <c r="I143" s="7"/>
       <c r="K143" s="7"/>
       <c r="L143" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M143" s="7"/>
@@ -4284,7 +4255,7 @@
     <row r="144">
       <c r="A144" s="6"/>
       <c r="B144" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F144" s="7"/>
@@ -4292,7 +4263,7 @@
       <c r="I144" s="7"/>
       <c r="K144" s="7"/>
       <c r="L144" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M144" s="7"/>
@@ -4301,7 +4272,7 @@
     <row r="145">
       <c r="A145" s="6"/>
       <c r="B145" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F145" s="7"/>
@@ -4309,7 +4280,7 @@
       <c r="I145" s="7"/>
       <c r="K145" s="7"/>
       <c r="L145" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M145" s="7"/>
@@ -4318,7 +4289,7 @@
     <row r="146">
       <c r="A146" s="6"/>
       <c r="B146" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F146" s="7"/>
@@ -4326,7 +4297,7 @@
       <c r="I146" s="7"/>
       <c r="K146" s="7"/>
       <c r="L146" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M146" s="7"/>
@@ -4335,7 +4306,7 @@
     <row r="147">
       <c r="A147" s="6"/>
       <c r="B147" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F147" s="7"/>
@@ -4343,7 +4314,7 @@
       <c r="I147" s="7"/>
       <c r="K147" s="7"/>
       <c r="L147" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M147" s="7"/>
@@ -4352,7 +4323,7 @@
     <row r="148">
       <c r="A148" s="6"/>
       <c r="B148" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F148" s="7"/>
@@ -4360,7 +4331,7 @@
       <c r="I148" s="7"/>
       <c r="K148" s="7"/>
       <c r="L148" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M148" s="7"/>
@@ -4369,7 +4340,7 @@
     <row r="149">
       <c r="A149" s="6"/>
       <c r="B149" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F149" s="7"/>
@@ -4377,7 +4348,7 @@
       <c r="I149" s="7"/>
       <c r="K149" s="7"/>
       <c r="L149" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M149" s="7"/>
@@ -4386,7 +4357,7 @@
     <row r="150">
       <c r="A150" s="6"/>
       <c r="B150" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F150" s="7"/>
@@ -4394,7 +4365,7 @@
       <c r="I150" s="7"/>
       <c r="K150" s="7"/>
       <c r="L150" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M150" s="7"/>
@@ -4403,7 +4374,7 @@
     <row r="151">
       <c r="A151" s="6"/>
       <c r="B151" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F151" s="7"/>
@@ -4411,7 +4382,7 @@
       <c r="I151" s="7"/>
       <c r="K151" s="7"/>
       <c r="L151" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M151" s="7"/>
@@ -4420,7 +4391,7 @@
     <row r="152">
       <c r="A152" s="6"/>
       <c r="B152" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F152" s="7"/>
@@ -4428,7 +4399,7 @@
       <c r="I152" s="7"/>
       <c r="K152" s="7"/>
       <c r="L152" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M152" s="7"/>
@@ -4437,7 +4408,7 @@
     <row r="153">
       <c r="A153" s="6"/>
       <c r="B153" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F153" s="7"/>
@@ -4445,7 +4416,7 @@
       <c r="I153" s="7"/>
       <c r="K153" s="7"/>
       <c r="L153" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M153" s="7"/>
@@ -4454,7 +4425,7 @@
     <row r="154">
       <c r="A154" s="6"/>
       <c r="B154" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F154" s="7"/>
@@ -4462,7 +4433,7 @@
       <c r="I154" s="7"/>
       <c r="K154" s="7"/>
       <c r="L154" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M154" s="7"/>
@@ -4471,7 +4442,7 @@
     <row r="155">
       <c r="A155" s="6"/>
       <c r="B155" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F155" s="7"/>
@@ -4479,7 +4450,7 @@
       <c r="I155" s="7"/>
       <c r="K155" s="7"/>
       <c r="L155" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M155" s="7"/>
@@ -4488,7 +4459,7 @@
     <row r="156">
       <c r="A156" s="6"/>
       <c r="B156" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F156" s="7"/>
@@ -4496,7 +4467,7 @@
       <c r="I156" s="7"/>
       <c r="K156" s="7"/>
       <c r="L156" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M156" s="7"/>
@@ -4505,7 +4476,7 @@
     <row r="157">
       <c r="A157" s="6"/>
       <c r="B157" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F157" s="7"/>
@@ -4513,7 +4484,7 @@
       <c r="I157" s="7"/>
       <c r="K157" s="7"/>
       <c r="L157" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M157" s="7"/>
@@ -4522,7 +4493,7 @@
     <row r="158">
       <c r="A158" s="6"/>
       <c r="B158" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F158" s="7"/>
@@ -4530,7 +4501,7 @@
       <c r="I158" s="7"/>
       <c r="K158" s="7"/>
       <c r="L158" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M158" s="7"/>
@@ -4539,7 +4510,7 @@
     <row r="159">
       <c r="A159" s="6"/>
       <c r="B159" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F159" s="7"/>
@@ -4547,7 +4518,7 @@
       <c r="I159" s="7"/>
       <c r="K159" s="7"/>
       <c r="L159" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M159" s="7"/>
@@ -4556,7 +4527,7 @@
     <row r="160">
       <c r="A160" s="6"/>
       <c r="B160" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F160" s="7"/>
@@ -4564,7 +4535,7 @@
       <c r="I160" s="7"/>
       <c r="K160" s="7"/>
       <c r="L160" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M160" s="7"/>
@@ -4573,7 +4544,7 @@
     <row r="161">
       <c r="A161" s="6"/>
       <c r="B161" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F161" s="7"/>
@@ -4581,7 +4552,7 @@
       <c r="I161" s="7"/>
       <c r="K161" s="7"/>
       <c r="L161" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M161" s="7"/>
@@ -4590,7 +4561,7 @@
     <row r="162">
       <c r="A162" s="6"/>
       <c r="B162" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F162" s="7"/>
@@ -4598,7 +4569,7 @@
       <c r="I162" s="7"/>
       <c r="K162" s="7"/>
       <c r="L162" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M162" s="7"/>
@@ -4607,7 +4578,7 @@
     <row r="163">
       <c r="A163" s="6"/>
       <c r="B163" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F163" s="7"/>
@@ -4615,7 +4586,7 @@
       <c r="I163" s="7"/>
       <c r="K163" s="7"/>
       <c r="L163" s="7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="M163" s="7"/>
@@ -4624,7 +4595,7 @@
     <row r="164">
       <c r="A164" s="6"/>
       <c r="B164" t="str">
-        <f t="shared" ref="B164:B227" si="7">IF(A164="","",WEEKNUM(A164,2))</f>
+        <f t="shared" ref="B164:B227" si="6">IF(A164="","",WEEKNUM(A164,2))</f>
         <v/>
       </c>
       <c r="F164" s="7"/>
@@ -4632,7 +4603,7 @@
       <c r="I164" s="7"/>
       <c r="K164" s="7"/>
       <c r="L164" s="7" t="str">
-        <f t="shared" ref="L164:L227" si="8">IF(OR(F164="",G164=""),"",F164*G164)</f>
+        <f t="shared" ref="L164:L227" si="7">IF(OR(F164="",G164=""),"",F164*G164)</f>
         <v/>
       </c>
       <c r="M164" s="7"/>
@@ -4641,7 +4612,7 @@
     <row r="165">
       <c r="A165" s="6"/>
       <c r="B165" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F165" s="7"/>
@@ -4649,7 +4620,7 @@
       <c r="I165" s="7"/>
       <c r="K165" s="7"/>
       <c r="L165" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M165" s="7"/>
@@ -4658,7 +4629,7 @@
     <row r="166">
       <c r="A166" s="6"/>
       <c r="B166" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F166" s="7"/>
@@ -4666,7 +4637,7 @@
       <c r="I166" s="7"/>
       <c r="K166" s="7"/>
       <c r="L166" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M166" s="7"/>
@@ -4675,7 +4646,7 @@
     <row r="167">
       <c r="A167" s="6"/>
       <c r="B167" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F167" s="7"/>
@@ -4683,7 +4654,7 @@
       <c r="I167" s="7"/>
       <c r="K167" s="7"/>
       <c r="L167" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M167" s="7"/>
@@ -4692,7 +4663,7 @@
     <row r="168">
       <c r="A168" s="6"/>
       <c r="B168" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F168" s="7"/>
@@ -4700,7 +4671,7 @@
       <c r="I168" s="7"/>
       <c r="K168" s="7"/>
       <c r="L168" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M168" s="7"/>
@@ -4709,7 +4680,7 @@
     <row r="169">
       <c r="A169" s="6"/>
       <c r="B169" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F169" s="7"/>
@@ -4717,7 +4688,7 @@
       <c r="I169" s="7"/>
       <c r="K169" s="7"/>
       <c r="L169" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M169" s="7"/>
@@ -4726,7 +4697,7 @@
     <row r="170">
       <c r="A170" s="6"/>
       <c r="B170" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F170" s="7"/>
@@ -4734,7 +4705,7 @@
       <c r="I170" s="7"/>
       <c r="K170" s="7"/>
       <c r="L170" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M170" s="7"/>
@@ -4743,7 +4714,7 @@
     <row r="171">
       <c r="A171" s="6"/>
       <c r="B171" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F171" s="7"/>
@@ -4751,7 +4722,7 @@
       <c r="I171" s="7"/>
       <c r="K171" s="7"/>
       <c r="L171" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M171" s="7"/>
@@ -4760,7 +4731,7 @@
     <row r="172">
       <c r="A172" s="6"/>
       <c r="B172" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F172" s="7"/>
@@ -4768,7 +4739,7 @@
       <c r="I172" s="7"/>
       <c r="K172" s="7"/>
       <c r="L172" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M172" s="7"/>
@@ -4777,7 +4748,7 @@
     <row r="173">
       <c r="A173" s="6"/>
       <c r="B173" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F173" s="7"/>
@@ -4785,7 +4756,7 @@
       <c r="I173" s="7"/>
       <c r="K173" s="7"/>
       <c r="L173" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M173" s="7"/>
@@ -4794,7 +4765,7 @@
     <row r="174">
       <c r="A174" s="6"/>
       <c r="B174" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F174" s="7"/>
@@ -4802,7 +4773,7 @@
       <c r="I174" s="7"/>
       <c r="K174" s="7"/>
       <c r="L174" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M174" s="7"/>
@@ -4811,7 +4782,7 @@
     <row r="175">
       <c r="A175" s="6"/>
       <c r="B175" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F175" s="7"/>
@@ -4819,7 +4790,7 @@
       <c r="I175" s="7"/>
       <c r="K175" s="7"/>
       <c r="L175" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M175" s="7"/>
@@ -4828,7 +4799,7 @@
     <row r="176">
       <c r="A176" s="6"/>
       <c r="B176" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F176" s="7"/>
@@ -4836,7 +4807,7 @@
       <c r="I176" s="7"/>
       <c r="K176" s="7"/>
       <c r="L176" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M176" s="7"/>
@@ -4845,7 +4816,7 @@
     <row r="177">
       <c r="A177" s="6"/>
       <c r="B177" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F177" s="7"/>
@@ -4853,7 +4824,7 @@
       <c r="I177" s="7"/>
       <c r="K177" s="7"/>
       <c r="L177" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M177" s="7"/>
@@ -4862,7 +4833,7 @@
     <row r="178">
       <c r="A178" s="6"/>
       <c r="B178" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F178" s="7"/>
@@ -4870,7 +4841,7 @@
       <c r="I178" s="7"/>
       <c r="K178" s="7"/>
       <c r="L178" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M178" s="7"/>
@@ -4879,7 +4850,7 @@
     <row r="179">
       <c r="A179" s="6"/>
       <c r="B179" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F179" s="7"/>
@@ -4887,7 +4858,7 @@
       <c r="I179" s="7"/>
       <c r="K179" s="7"/>
       <c r="L179" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M179" s="7"/>
@@ -4896,7 +4867,7 @@
     <row r="180">
       <c r="A180" s="6"/>
       <c r="B180" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F180" s="7"/>
@@ -4904,7 +4875,7 @@
       <c r="I180" s="7"/>
       <c r="K180" s="7"/>
       <c r="L180" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M180" s="7"/>
@@ -4913,7 +4884,7 @@
     <row r="181">
       <c r="A181" s="6"/>
       <c r="B181" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F181" s="7"/>
@@ -4921,7 +4892,7 @@
       <c r="I181" s="7"/>
       <c r="K181" s="7"/>
       <c r="L181" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M181" s="7"/>
@@ -4930,7 +4901,7 @@
     <row r="182">
       <c r="A182" s="6"/>
       <c r="B182" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F182" s="7"/>
@@ -4938,7 +4909,7 @@
       <c r="I182" s="7"/>
       <c r="K182" s="7"/>
       <c r="L182" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M182" s="7"/>
@@ -4947,7 +4918,7 @@
     <row r="183">
       <c r="A183" s="6"/>
       <c r="B183" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F183" s="7"/>
@@ -4955,7 +4926,7 @@
       <c r="I183" s="7"/>
       <c r="K183" s="7"/>
       <c r="L183" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M183" s="7"/>
@@ -4964,7 +4935,7 @@
     <row r="184">
       <c r="A184" s="6"/>
       <c r="B184" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F184" s="7"/>
@@ -4972,7 +4943,7 @@
       <c r="I184" s="7"/>
       <c r="K184" s="7"/>
       <c r="L184" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M184" s="7"/>
@@ -4981,7 +4952,7 @@
     <row r="185">
       <c r="A185" s="6"/>
       <c r="B185" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F185" s="7"/>
@@ -4989,7 +4960,7 @@
       <c r="I185" s="7"/>
       <c r="K185" s="7"/>
       <c r="L185" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M185" s="7"/>
@@ -4998,7 +4969,7 @@
     <row r="186">
       <c r="A186" s="6"/>
       <c r="B186" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F186" s="7"/>
@@ -5006,7 +4977,7 @@
       <c r="I186" s="7"/>
       <c r="K186" s="7"/>
       <c r="L186" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M186" s="7"/>
@@ -5015,7 +4986,7 @@
     <row r="187">
       <c r="A187" s="6"/>
       <c r="B187" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F187" s="7"/>
@@ -5023,7 +4994,7 @@
       <c r="I187" s="7"/>
       <c r="K187" s="7"/>
       <c r="L187" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M187" s="7"/>
@@ -5032,7 +5003,7 @@
     <row r="188">
       <c r="A188" s="6"/>
       <c r="B188" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F188" s="7"/>
@@ -5040,7 +5011,7 @@
       <c r="I188" s="7"/>
       <c r="K188" s="7"/>
       <c r="L188" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M188" s="7"/>
@@ -5049,7 +5020,7 @@
     <row r="189">
       <c r="A189" s="6"/>
       <c r="B189" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F189" s="7"/>
@@ -5057,7 +5028,7 @@
       <c r="I189" s="7"/>
       <c r="K189" s="7"/>
       <c r="L189" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M189" s="7"/>
@@ -5066,7 +5037,7 @@
     <row r="190">
       <c r="A190" s="6"/>
       <c r="B190" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F190" s="7"/>
@@ -5074,7 +5045,7 @@
       <c r="I190" s="7"/>
       <c r="K190" s="7"/>
       <c r="L190" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M190" s="7"/>
@@ -5083,7 +5054,7 @@
     <row r="191">
       <c r="A191" s="6"/>
       <c r="B191" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F191" s="7"/>
@@ -5091,7 +5062,7 @@
       <c r="I191" s="7"/>
       <c r="K191" s="7"/>
       <c r="L191" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M191" s="7"/>
@@ -5100,7 +5071,7 @@
     <row r="192">
       <c r="A192" s="6"/>
       <c r="B192" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F192" s="7"/>
@@ -5108,7 +5079,7 @@
       <c r="I192" s="7"/>
       <c r="K192" s="7"/>
       <c r="L192" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M192" s="7"/>
@@ -5117,7 +5088,7 @@
     <row r="193">
       <c r="A193" s="6"/>
       <c r="B193" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F193" s="7"/>
@@ -5125,7 +5096,7 @@
       <c r="I193" s="7"/>
       <c r="K193" s="7"/>
       <c r="L193" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M193" s="7"/>
@@ -5134,7 +5105,7 @@
     <row r="194">
       <c r="A194" s="6"/>
       <c r="B194" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F194" s="7"/>
@@ -5142,7 +5113,7 @@
       <c r="I194" s="7"/>
       <c r="K194" s="7"/>
       <c r="L194" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M194" s="7"/>
@@ -5151,7 +5122,7 @@
     <row r="195">
       <c r="A195" s="6"/>
       <c r="B195" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F195" s="7"/>
@@ -5159,7 +5130,7 @@
       <c r="I195" s="7"/>
       <c r="K195" s="7"/>
       <c r="L195" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M195" s="7"/>
@@ -5168,7 +5139,7 @@
     <row r="196">
       <c r="A196" s="6"/>
       <c r="B196" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F196" s="7"/>
@@ -5176,7 +5147,7 @@
       <c r="I196" s="7"/>
       <c r="K196" s="7"/>
       <c r="L196" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M196" s="7"/>
@@ -5185,7 +5156,7 @@
     <row r="197">
       <c r="A197" s="6"/>
       <c r="B197" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F197" s="7"/>
@@ -5193,7 +5164,7 @@
       <c r="I197" s="7"/>
       <c r="K197" s="7"/>
       <c r="L197" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M197" s="7"/>
@@ -5202,7 +5173,7 @@
     <row r="198">
       <c r="A198" s="6"/>
       <c r="B198" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F198" s="7"/>
@@ -5210,7 +5181,7 @@
       <c r="I198" s="7"/>
       <c r="K198" s="7"/>
       <c r="L198" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M198" s="7"/>
@@ -5219,7 +5190,7 @@
     <row r="199">
       <c r="A199" s="6"/>
       <c r="B199" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F199" s="7"/>
@@ -5227,7 +5198,7 @@
       <c r="I199" s="7"/>
       <c r="K199" s="7"/>
       <c r="L199" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M199" s="7"/>
@@ -5236,7 +5207,7 @@
     <row r="200">
       <c r="A200" s="6"/>
       <c r="B200" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F200" s="7"/>
@@ -5244,7 +5215,7 @@
       <c r="I200" s="7"/>
       <c r="K200" s="7"/>
       <c r="L200" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M200" s="7"/>
@@ -5253,7 +5224,7 @@
     <row r="201">
       <c r="A201" s="6"/>
       <c r="B201" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F201" s="7"/>
@@ -5261,7 +5232,7 @@
       <c r="I201" s="7"/>
       <c r="K201" s="7"/>
       <c r="L201" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M201" s="7"/>
@@ -5270,7 +5241,7 @@
     <row r="202">
       <c r="A202" s="6"/>
       <c r="B202" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F202" s="7"/>
@@ -5278,7 +5249,7 @@
       <c r="I202" s="7"/>
       <c r="K202" s="7"/>
       <c r="L202" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M202" s="7"/>
@@ -5287,7 +5258,7 @@
     <row r="203">
       <c r="A203" s="6"/>
       <c r="B203" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F203" s="7"/>
@@ -5295,7 +5266,7 @@
       <c r="I203" s="7"/>
       <c r="K203" s="7"/>
       <c r="L203" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M203" s="7"/>
@@ -5304,7 +5275,7 @@
     <row r="204">
       <c r="A204" s="6"/>
       <c r="B204" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F204" s="7"/>
@@ -5312,7 +5283,7 @@
       <c r="I204" s="7"/>
       <c r="K204" s="7"/>
       <c r="L204" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M204" s="7"/>
@@ -5321,7 +5292,7 @@
     <row r="205">
       <c r="A205" s="6"/>
       <c r="B205" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F205" s="7"/>
@@ -5329,7 +5300,7 @@
       <c r="I205" s="7"/>
       <c r="K205" s="7"/>
       <c r="L205" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M205" s="7"/>
@@ -5338,7 +5309,7 @@
     <row r="206">
       <c r="A206" s="6"/>
       <c r="B206" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F206" s="7"/>
@@ -5346,7 +5317,7 @@
       <c r="I206" s="7"/>
       <c r="K206" s="7"/>
       <c r="L206" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M206" s="7"/>
@@ -5355,7 +5326,7 @@
     <row r="207">
       <c r="A207" s="6"/>
       <c r="B207" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F207" s="7"/>
@@ -5363,7 +5334,7 @@
       <c r="I207" s="7"/>
       <c r="K207" s="7"/>
       <c r="L207" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M207" s="7"/>
@@ -5372,7 +5343,7 @@
     <row r="208">
       <c r="A208" s="6"/>
       <c r="B208" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F208" s="7"/>
@@ -5380,7 +5351,7 @@
       <c r="I208" s="7"/>
       <c r="K208" s="7"/>
       <c r="L208" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M208" s="7"/>
@@ -5389,7 +5360,7 @@
     <row r="209">
       <c r="A209" s="6"/>
       <c r="B209" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F209" s="7"/>
@@ -5397,7 +5368,7 @@
       <c r="I209" s="7"/>
       <c r="K209" s="7"/>
       <c r="L209" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M209" s="7"/>
@@ -5406,7 +5377,7 @@
     <row r="210">
       <c r="A210" s="6"/>
       <c r="B210" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F210" s="7"/>
@@ -5414,7 +5385,7 @@
       <c r="I210" s="7"/>
       <c r="K210" s="7"/>
       <c r="L210" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M210" s="7"/>
@@ -5423,7 +5394,7 @@
     <row r="211">
       <c r="A211" s="6"/>
       <c r="B211" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F211" s="7"/>
@@ -5431,7 +5402,7 @@
       <c r="I211" s="7"/>
       <c r="K211" s="7"/>
       <c r="L211" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M211" s="7"/>
@@ -5440,7 +5411,7 @@
     <row r="212">
       <c r="A212" s="6"/>
       <c r="B212" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F212" s="7"/>
@@ -5448,7 +5419,7 @@
       <c r="I212" s="7"/>
       <c r="K212" s="7"/>
       <c r="L212" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M212" s="7"/>
@@ -5457,7 +5428,7 @@
     <row r="213">
       <c r="A213" s="6"/>
       <c r="B213" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F213" s="7"/>
@@ -5465,7 +5436,7 @@
       <c r="I213" s="7"/>
       <c r="K213" s="7"/>
       <c r="L213" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M213" s="7"/>
@@ -5474,7 +5445,7 @@
     <row r="214">
       <c r="A214" s="6"/>
       <c r="B214" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F214" s="7"/>
@@ -5482,7 +5453,7 @@
       <c r="I214" s="7"/>
       <c r="K214" s="7"/>
       <c r="L214" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M214" s="7"/>
@@ -5491,7 +5462,7 @@
     <row r="215">
       <c r="A215" s="6"/>
       <c r="B215" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F215" s="7"/>
@@ -5499,7 +5470,7 @@
       <c r="I215" s="7"/>
       <c r="K215" s="7"/>
       <c r="L215" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M215" s="7"/>
@@ -5508,7 +5479,7 @@
     <row r="216">
       <c r="A216" s="6"/>
       <c r="B216" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F216" s="7"/>
@@ -5516,7 +5487,7 @@
       <c r="I216" s="7"/>
       <c r="K216" s="7"/>
       <c r="L216" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M216" s="7"/>
@@ -5525,7 +5496,7 @@
     <row r="217">
       <c r="A217" s="6"/>
       <c r="B217" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F217" s="7"/>
@@ -5533,7 +5504,7 @@
       <c r="I217" s="7"/>
       <c r="K217" s="7"/>
       <c r="L217" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M217" s="7"/>
@@ -5542,7 +5513,7 @@
     <row r="218">
       <c r="A218" s="6"/>
       <c r="B218" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F218" s="7"/>
@@ -5550,7 +5521,7 @@
       <c r="I218" s="7"/>
       <c r="K218" s="7"/>
       <c r="L218" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M218" s="7"/>
@@ -5559,7 +5530,7 @@
     <row r="219">
       <c r="A219" s="6"/>
       <c r="B219" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F219" s="7"/>
@@ -5567,7 +5538,7 @@
       <c r="I219" s="7"/>
       <c r="K219" s="7"/>
       <c r="L219" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M219" s="7"/>
@@ -5576,7 +5547,7 @@
     <row r="220">
       <c r="A220" s="6"/>
       <c r="B220" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F220" s="7"/>
@@ -5584,7 +5555,7 @@
       <c r="I220" s="7"/>
       <c r="K220" s="7"/>
       <c r="L220" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M220" s="7"/>
@@ -5593,7 +5564,7 @@
     <row r="221">
       <c r="A221" s="6"/>
       <c r="B221" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F221" s="7"/>
@@ -5601,7 +5572,7 @@
       <c r="I221" s="7"/>
       <c r="K221" s="7"/>
       <c r="L221" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M221" s="7"/>
@@ -5610,7 +5581,7 @@
     <row r="222">
       <c r="A222" s="6"/>
       <c r="B222" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F222" s="7"/>
@@ -5618,7 +5589,7 @@
       <c r="I222" s="7"/>
       <c r="K222" s="7"/>
       <c r="L222" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M222" s="7"/>
@@ -5627,7 +5598,7 @@
     <row r="223">
       <c r="A223" s="6"/>
       <c r="B223" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F223" s="7"/>
@@ -5635,7 +5606,7 @@
       <c r="I223" s="7"/>
       <c r="K223" s="7"/>
       <c r="L223" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M223" s="7"/>
@@ -5644,7 +5615,7 @@
     <row r="224">
       <c r="A224" s="6"/>
       <c r="B224" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F224" s="7"/>
@@ -5652,7 +5623,7 @@
       <c r="I224" s="7"/>
       <c r="K224" s="7"/>
       <c r="L224" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M224" s="7"/>
@@ -5661,7 +5632,7 @@
     <row r="225">
       <c r="A225" s="6"/>
       <c r="B225" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F225" s="7"/>
@@ -5669,7 +5640,7 @@
       <c r="I225" s="7"/>
       <c r="K225" s="7"/>
       <c r="L225" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M225" s="7"/>
@@ -5678,7 +5649,7 @@
     <row r="226">
       <c r="A226" s="6"/>
       <c r="B226" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F226" s="7"/>
@@ -5686,7 +5657,7 @@
       <c r="I226" s="7"/>
       <c r="K226" s="7"/>
       <c r="L226" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M226" s="7"/>
@@ -5695,7 +5666,7 @@
     <row r="227">
       <c r="A227" s="6"/>
       <c r="B227" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="F227" s="7"/>
@@ -5703,7 +5674,7 @@
       <c r="I227" s="7"/>
       <c r="K227" s="7"/>
       <c r="L227" s="7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="M227" s="7"/>
@@ -5712,7 +5683,7 @@
     <row r="228">
       <c r="A228" s="6"/>
       <c r="B228" t="str">
-        <f t="shared" ref="B228:B291" si="9">IF(A228="","",WEEKNUM(A228,2))</f>
+        <f t="shared" ref="B228:B291" si="8">IF(A228="","",WEEKNUM(A228,2))</f>
         <v/>
       </c>
       <c r="F228" s="7"/>
@@ -5720,7 +5691,7 @@
       <c r="I228" s="7"/>
       <c r="K228" s="7"/>
       <c r="L228" s="7" t="str">
-        <f t="shared" ref="L228:L291" si="10">IF(OR(F228="",G228=""),"",F228*G228)</f>
+        <f t="shared" ref="L228:L291" si="9">IF(OR(F228="",G228=""),"",F228*G228)</f>
         <v/>
       </c>
       <c r="M228" s="7"/>
@@ -5729,7 +5700,7 @@
     <row r="229">
       <c r="A229" s="6"/>
       <c r="B229" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F229" s="7"/>
@@ -5737,7 +5708,7 @@
       <c r="I229" s="7"/>
       <c r="K229" s="7"/>
       <c r="L229" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M229" s="7"/>
@@ -5746,7 +5717,7 @@
     <row r="230">
       <c r="A230" s="6"/>
       <c r="B230" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F230" s="7"/>
@@ -5754,7 +5725,7 @@
       <c r="I230" s="7"/>
       <c r="K230" s="7"/>
       <c r="L230" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M230" s="7"/>
@@ -5763,7 +5734,7 @@
     <row r="231">
       <c r="A231" s="6"/>
       <c r="B231" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F231" s="7"/>
@@ -5771,7 +5742,7 @@
       <c r="I231" s="7"/>
       <c r="K231" s="7"/>
       <c r="L231" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M231" s="7"/>
@@ -5780,7 +5751,7 @@
     <row r="232">
       <c r="A232" s="6"/>
       <c r="B232" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F232" s="7"/>
@@ -5788,7 +5759,7 @@
       <c r="I232" s="7"/>
       <c r="K232" s="7"/>
       <c r="L232" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M232" s="7"/>
@@ -5797,7 +5768,7 @@
     <row r="233">
       <c r="A233" s="6"/>
       <c r="B233" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F233" s="7"/>
@@ -5805,7 +5776,7 @@
       <c r="I233" s="7"/>
       <c r="K233" s="7"/>
       <c r="L233" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M233" s="7"/>
@@ -5814,7 +5785,7 @@
     <row r="234">
       <c r="A234" s="6"/>
       <c r="B234" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F234" s="7"/>
@@ -5822,7 +5793,7 @@
       <c r="I234" s="7"/>
       <c r="K234" s="7"/>
       <c r="L234" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M234" s="7"/>
@@ -5831,7 +5802,7 @@
     <row r="235">
       <c r="A235" s="6"/>
       <c r="B235" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F235" s="7"/>
@@ -5839,7 +5810,7 @@
       <c r="I235" s="7"/>
       <c r="K235" s="7"/>
       <c r="L235" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M235" s="7"/>
@@ -5848,7 +5819,7 @@
     <row r="236">
       <c r="A236" s="6"/>
       <c r="B236" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F236" s="7"/>
@@ -5856,7 +5827,7 @@
       <c r="I236" s="7"/>
       <c r="K236" s="7"/>
       <c r="L236" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M236" s="7"/>
@@ -5865,7 +5836,7 @@
     <row r="237">
       <c r="A237" s="6"/>
       <c r="B237" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F237" s="7"/>
@@ -5873,7 +5844,7 @@
       <c r="I237" s="7"/>
       <c r="K237" s="7"/>
       <c r="L237" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M237" s="7"/>
@@ -5882,7 +5853,7 @@
     <row r="238">
       <c r="A238" s="6"/>
       <c r="B238" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F238" s="7"/>
@@ -5890,7 +5861,7 @@
       <c r="I238" s="7"/>
       <c r="K238" s="7"/>
       <c r="L238" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M238" s="7"/>
@@ -5899,7 +5870,7 @@
     <row r="239">
       <c r="A239" s="6"/>
       <c r="B239" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F239" s="7"/>
@@ -5907,7 +5878,7 @@
       <c r="I239" s="7"/>
       <c r="K239" s="7"/>
       <c r="L239" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M239" s="7"/>
@@ -5916,7 +5887,7 @@
     <row r="240">
       <c r="A240" s="6"/>
       <c r="B240" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F240" s="7"/>
@@ -5924,7 +5895,7 @@
       <c r="I240" s="7"/>
       <c r="K240" s="7"/>
       <c r="L240" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M240" s="7"/>
@@ -5933,7 +5904,7 @@
     <row r="241">
       <c r="A241" s="6"/>
       <c r="B241" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F241" s="7"/>
@@ -5941,7 +5912,7 @@
       <c r="I241" s="7"/>
       <c r="K241" s="7"/>
       <c r="L241" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M241" s="7"/>
@@ -5950,7 +5921,7 @@
     <row r="242">
       <c r="A242" s="6"/>
       <c r="B242" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F242" s="7"/>
@@ -5958,7 +5929,7 @@
       <c r="I242" s="7"/>
       <c r="K242" s="7"/>
       <c r="L242" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M242" s="7"/>
@@ -5967,7 +5938,7 @@
     <row r="243">
       <c r="A243" s="6"/>
       <c r="B243" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F243" s="7"/>
@@ -5975,7 +5946,7 @@
       <c r="I243" s="7"/>
       <c r="K243" s="7"/>
       <c r="L243" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M243" s="7"/>
@@ -5984,7 +5955,7 @@
     <row r="244">
       <c r="A244" s="6"/>
       <c r="B244" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F244" s="7"/>
@@ -5992,7 +5963,7 @@
       <c r="I244" s="7"/>
       <c r="K244" s="7"/>
       <c r="L244" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M244" s="7"/>
@@ -6001,7 +5972,7 @@
     <row r="245">
       <c r="A245" s="6"/>
       <c r="B245" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F245" s="7"/>
@@ -6009,7 +5980,7 @@
       <c r="I245" s="7"/>
       <c r="K245" s="7"/>
       <c r="L245" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M245" s="7"/>
@@ -6018,7 +5989,7 @@
     <row r="246">
       <c r="A246" s="6"/>
       <c r="B246" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F246" s="7"/>
@@ -6026,7 +5997,7 @@
       <c r="I246" s="7"/>
       <c r="K246" s="7"/>
       <c r="L246" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M246" s="7"/>
@@ -6035,7 +6006,7 @@
     <row r="247">
       <c r="A247" s="6"/>
       <c r="B247" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F247" s="7"/>
@@ -6043,7 +6014,7 @@
       <c r="I247" s="7"/>
       <c r="K247" s="7"/>
       <c r="L247" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M247" s="7"/>
@@ -6052,7 +6023,7 @@
     <row r="248">
       <c r="A248" s="6"/>
       <c r="B248" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F248" s="7"/>
@@ -6060,7 +6031,7 @@
       <c r="I248" s="7"/>
       <c r="K248" s="7"/>
       <c r="L248" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M248" s="7"/>
@@ -6069,7 +6040,7 @@
     <row r="249">
       <c r="A249" s="6"/>
       <c r="B249" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F249" s="7"/>
@@ -6077,7 +6048,7 @@
       <c r="I249" s="7"/>
       <c r="K249" s="7"/>
       <c r="L249" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M249" s="7"/>
@@ -6086,7 +6057,7 @@
     <row r="250">
       <c r="A250" s="6"/>
       <c r="B250" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F250" s="7"/>
@@ -6094,7 +6065,7 @@
       <c r="I250" s="7"/>
       <c r="K250" s="7"/>
       <c r="L250" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M250" s="7"/>
@@ -6103,7 +6074,7 @@
     <row r="251">
       <c r="A251" s="6"/>
       <c r="B251" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F251" s="7"/>
@@ -6111,7 +6082,7 @@
       <c r="I251" s="7"/>
       <c r="K251" s="7"/>
       <c r="L251" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M251" s="7"/>
@@ -6120,7 +6091,7 @@
     <row r="252">
       <c r="A252" s="6"/>
       <c r="B252" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F252" s="7"/>
@@ -6128,7 +6099,7 @@
       <c r="I252" s="7"/>
       <c r="K252" s="7"/>
       <c r="L252" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M252" s="7"/>
@@ -6137,7 +6108,7 @@
     <row r="253">
       <c r="A253" s="6"/>
       <c r="B253" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F253" s="7"/>
@@ -6145,7 +6116,7 @@
       <c r="I253" s="7"/>
       <c r="K253" s="7"/>
       <c r="L253" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M253" s="7"/>
@@ -6154,7 +6125,7 @@
     <row r="254">
       <c r="A254" s="6"/>
       <c r="B254" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F254" s="7"/>
@@ -6162,7 +6133,7 @@
       <c r="I254" s="7"/>
       <c r="K254" s="7"/>
       <c r="L254" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M254" s="7"/>
@@ -6171,7 +6142,7 @@
     <row r="255">
       <c r="A255" s="6"/>
       <c r="B255" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F255" s="7"/>
@@ -6179,7 +6150,7 @@
       <c r="I255" s="7"/>
       <c r="K255" s="7"/>
       <c r="L255" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M255" s="7"/>
@@ -6188,7 +6159,7 @@
     <row r="256">
       <c r="A256" s="6"/>
       <c r="B256" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F256" s="7"/>
@@ -6196,7 +6167,7 @@
       <c r="I256" s="7"/>
       <c r="K256" s="7"/>
       <c r="L256" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M256" s="7"/>
@@ -6205,7 +6176,7 @@
     <row r="257">
       <c r="A257" s="6"/>
       <c r="B257" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F257" s="7"/>
@@ -6213,7 +6184,7 @@
       <c r="I257" s="7"/>
       <c r="K257" s="7"/>
       <c r="L257" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M257" s="7"/>
@@ -6222,7 +6193,7 @@
     <row r="258">
       <c r="A258" s="6"/>
       <c r="B258" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F258" s="7"/>
@@ -6230,7 +6201,7 @@
       <c r="I258" s="7"/>
       <c r="K258" s="7"/>
       <c r="L258" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M258" s="7"/>
@@ -6239,7 +6210,7 @@
     <row r="259">
       <c r="A259" s="6"/>
       <c r="B259" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F259" s="7"/>
@@ -6247,7 +6218,7 @@
       <c r="I259" s="7"/>
       <c r="K259" s="7"/>
       <c r="L259" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M259" s="7"/>
@@ -6256,7 +6227,7 @@
     <row r="260">
       <c r="A260" s="6"/>
       <c r="B260" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F260" s="7"/>
@@ -6264,7 +6235,7 @@
       <c r="I260" s="7"/>
       <c r="K260" s="7"/>
       <c r="L260" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M260" s="7"/>
@@ -6273,7 +6244,7 @@
     <row r="261">
       <c r="A261" s="6"/>
       <c r="B261" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F261" s="7"/>
@@ -6281,7 +6252,7 @@
       <c r="I261" s="7"/>
       <c r="K261" s="7"/>
       <c r="L261" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M261" s="7"/>
@@ -6290,7 +6261,7 @@
     <row r="262">
       <c r="A262" s="6"/>
       <c r="B262" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F262" s="7"/>
@@ -6298,7 +6269,7 @@
       <c r="I262" s="7"/>
       <c r="K262" s="7"/>
       <c r="L262" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M262" s="7"/>
@@ -6307,7 +6278,7 @@
     <row r="263">
       <c r="A263" s="6"/>
       <c r="B263" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F263" s="7"/>
@@ -6315,7 +6286,7 @@
       <c r="I263" s="7"/>
       <c r="K263" s="7"/>
       <c r="L263" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M263" s="7"/>
@@ -6324,7 +6295,7 @@
     <row r="264">
       <c r="A264" s="6"/>
       <c r="B264" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F264" s="7"/>
@@ -6332,7 +6303,7 @@
       <c r="I264" s="7"/>
       <c r="K264" s="7"/>
       <c r="L264" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M264" s="7"/>
@@ -6341,7 +6312,7 @@
     <row r="265">
       <c r="A265" s="6"/>
       <c r="B265" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F265" s="7"/>
@@ -6349,7 +6320,7 @@
       <c r="I265" s="7"/>
       <c r="K265" s="7"/>
       <c r="L265" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M265" s="7"/>
@@ -6358,7 +6329,7 @@
     <row r="266">
       <c r="A266" s="6"/>
       <c r="B266" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F266" s="7"/>
@@ -6366,7 +6337,7 @@
       <c r="I266" s="7"/>
       <c r="K266" s="7"/>
       <c r="L266" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M266" s="7"/>
@@ -6375,7 +6346,7 @@
     <row r="267">
       <c r="A267" s="6"/>
       <c r="B267" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F267" s="7"/>
@@ -6383,7 +6354,7 @@
       <c r="I267" s="7"/>
       <c r="K267" s="7"/>
       <c r="L267" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M267" s="7"/>
@@ -6392,7 +6363,7 @@
     <row r="268">
       <c r="A268" s="6"/>
       <c r="B268" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F268" s="7"/>
@@ -6400,7 +6371,7 @@
       <c r="I268" s="7"/>
       <c r="K268" s="7"/>
       <c r="L268" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M268" s="7"/>
@@ -6409,7 +6380,7 @@
     <row r="269">
       <c r="A269" s="6"/>
       <c r="B269" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F269" s="7"/>
@@ -6417,7 +6388,7 @@
       <c r="I269" s="7"/>
       <c r="K269" s="7"/>
       <c r="L269" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M269" s="7"/>
@@ -6426,7 +6397,7 @@
     <row r="270">
       <c r="A270" s="6"/>
       <c r="B270" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F270" s="7"/>
@@ -6434,7 +6405,7 @@
       <c r="I270" s="7"/>
       <c r="K270" s="7"/>
       <c r="L270" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M270" s="7"/>
@@ -6443,7 +6414,7 @@
     <row r="271">
       <c r="A271" s="6"/>
       <c r="B271" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F271" s="7"/>
@@ -6451,7 +6422,7 @@
       <c r="I271" s="7"/>
       <c r="K271" s="7"/>
       <c r="L271" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M271" s="7"/>
@@ -6460,7 +6431,7 @@
     <row r="272">
       <c r="A272" s="6"/>
       <c r="B272" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F272" s="7"/>
@@ -6468,7 +6439,7 @@
       <c r="I272" s="7"/>
       <c r="K272" s="7"/>
       <c r="L272" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M272" s="7"/>
@@ -6477,7 +6448,7 @@
     <row r="273">
       <c r="A273" s="6"/>
       <c r="B273" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F273" s="7"/>
@@ -6485,7 +6456,7 @@
       <c r="I273" s="7"/>
       <c r="K273" s="7"/>
       <c r="L273" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M273" s="7"/>
@@ -6494,7 +6465,7 @@
     <row r="274">
       <c r="A274" s="6"/>
       <c r="B274" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F274" s="7"/>
@@ -6502,7 +6473,7 @@
       <c r="I274" s="7"/>
       <c r="K274" s="7"/>
       <c r="L274" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M274" s="7"/>
@@ -6511,7 +6482,7 @@
     <row r="275">
       <c r="A275" s="6"/>
       <c r="B275" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F275" s="7"/>
@@ -6519,7 +6490,7 @@
       <c r="I275" s="7"/>
       <c r="K275" s="7"/>
       <c r="L275" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M275" s="7"/>
@@ -6528,7 +6499,7 @@
     <row r="276">
       <c r="A276" s="6"/>
       <c r="B276" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F276" s="7"/>
@@ -6536,7 +6507,7 @@
       <c r="I276" s="7"/>
       <c r="K276" s="7"/>
       <c r="L276" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M276" s="7"/>
@@ -6545,7 +6516,7 @@
     <row r="277">
       <c r="A277" s="6"/>
       <c r="B277" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F277" s="7"/>
@@ -6553,7 +6524,7 @@
       <c r="I277" s="7"/>
       <c r="K277" s="7"/>
       <c r="L277" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M277" s="7"/>
@@ -6562,7 +6533,7 @@
     <row r="278">
       <c r="A278" s="6"/>
       <c r="B278" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F278" s="7"/>
@@ -6570,7 +6541,7 @@
       <c r="I278" s="7"/>
       <c r="K278" s="7"/>
       <c r="L278" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M278" s="7"/>
@@ -6579,7 +6550,7 @@
     <row r="279">
       <c r="A279" s="6"/>
       <c r="B279" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F279" s="7"/>
@@ -6587,7 +6558,7 @@
       <c r="I279" s="7"/>
       <c r="K279" s="7"/>
       <c r="L279" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M279" s="7"/>
@@ -6596,7 +6567,7 @@
     <row r="280">
       <c r="A280" s="6"/>
       <c r="B280" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F280" s="7"/>
@@ -6604,7 +6575,7 @@
       <c r="I280" s="7"/>
       <c r="K280" s="7"/>
       <c r="L280" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M280" s="7"/>
@@ -6613,7 +6584,7 @@
     <row r="281">
       <c r="A281" s="6"/>
       <c r="B281" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F281" s="7"/>
@@ -6621,7 +6592,7 @@
       <c r="I281" s="7"/>
       <c r="K281" s="7"/>
       <c r="L281" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M281" s="7"/>
@@ -6630,7 +6601,7 @@
     <row r="282">
       <c r="A282" s="6"/>
       <c r="B282" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F282" s="7"/>
@@ -6638,7 +6609,7 @@
       <c r="I282" s="7"/>
       <c r="K282" s="7"/>
       <c r="L282" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M282" s="7"/>
@@ -6647,7 +6618,7 @@
     <row r="283">
       <c r="A283" s="6"/>
       <c r="B283" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F283" s="7"/>
@@ -6655,7 +6626,7 @@
       <c r="I283" s="7"/>
       <c r="K283" s="7"/>
       <c r="L283" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M283" s="7"/>
@@ -6664,7 +6635,7 @@
     <row r="284">
       <c r="A284" s="6"/>
       <c r="B284" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F284" s="7"/>
@@ -6672,7 +6643,7 @@
       <c r="I284" s="7"/>
       <c r="K284" s="7"/>
       <c r="L284" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M284" s="7"/>
@@ -6681,7 +6652,7 @@
     <row r="285">
       <c r="A285" s="6"/>
       <c r="B285" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F285" s="7"/>
@@ -6689,7 +6660,7 @@
       <c r="I285" s="7"/>
       <c r="K285" s="7"/>
       <c r="L285" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M285" s="7"/>
@@ -6698,7 +6669,7 @@
     <row r="286">
       <c r="A286" s="6"/>
       <c r="B286" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F286" s="7"/>
@@ -6706,7 +6677,7 @@
       <c r="I286" s="7"/>
       <c r="K286" s="7"/>
       <c r="L286" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M286" s="7"/>
@@ -6715,7 +6686,7 @@
     <row r="287">
       <c r="A287" s="6"/>
       <c r="B287" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F287" s="7"/>
@@ -6723,7 +6694,7 @@
       <c r="I287" s="7"/>
       <c r="K287" s="7"/>
       <c r="L287" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M287" s="7"/>
@@ -6732,7 +6703,7 @@
     <row r="288">
       <c r="A288" s="6"/>
       <c r="B288" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F288" s="7"/>
@@ -6740,7 +6711,7 @@
       <c r="I288" s="7"/>
       <c r="K288" s="7"/>
       <c r="L288" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M288" s="7"/>
@@ -6749,7 +6720,7 @@
     <row r="289">
       <c r="A289" s="6"/>
       <c r="B289" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F289" s="7"/>
@@ -6757,7 +6728,7 @@
       <c r="I289" s="7"/>
       <c r="K289" s="7"/>
       <c r="L289" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M289" s="7"/>
@@ -6766,7 +6737,7 @@
     <row r="290">
       <c r="A290" s="6"/>
       <c r="B290" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F290" s="7"/>
@@ -6774,7 +6745,7 @@
       <c r="I290" s="7"/>
       <c r="K290" s="7"/>
       <c r="L290" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M290" s="7"/>
@@ -6783,7 +6754,7 @@
     <row r="291">
       <c r="A291" s="6"/>
       <c r="B291" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="F291" s="7"/>
@@ -6791,7 +6762,7 @@
       <c r="I291" s="7"/>
       <c r="K291" s="7"/>
       <c r="L291" s="7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="M291" s="7"/>
@@ -6800,7 +6771,7 @@
     <row r="292">
       <c r="A292" s="6"/>
       <c r="B292" t="str">
-        <f t="shared" ref="B292:B303" si="11">IF(A292="","",WEEKNUM(A292,2))</f>
+        <f t="shared" ref="B292:B303" si="10">IF(A292="","",WEEKNUM(A292,2))</f>
         <v/>
       </c>
       <c r="F292" s="7"/>
@@ -6808,7 +6779,7 @@
       <c r="I292" s="7"/>
       <c r="K292" s="7"/>
       <c r="L292" s="7" t="str">
-        <f t="shared" ref="L292:L303" si="12">IF(OR(F292="",G292=""),"",F292*G292)</f>
+        <f t="shared" ref="L292:L303" si="11">IF(OR(F292="",G292=""),"",F292*G292)</f>
         <v/>
       </c>
       <c r="M292" s="7"/>
@@ -6817,7 +6788,7 @@
     <row r="293">
       <c r="A293" s="6"/>
       <c r="B293" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="F293" s="7"/>
@@ -6825,7 +6796,7 @@
       <c r="I293" s="7"/>
       <c r="K293" s="7"/>
       <c r="L293" s="7" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="M293" s="7"/>
@@ -6834,7 +6805,7 @@
     <row r="294">
       <c r="A294" s="6"/>
       <c r="B294" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="F294" s="7"/>
@@ -6842,7 +6813,7 @@
       <c r="I294" s="7"/>
       <c r="K294" s="7"/>
       <c r="L294" s="7" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="M294" s="7"/>
@@ -6851,7 +6822,7 @@
     <row r="295">
       <c r="A295" s="6"/>
       <c r="B295" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="F295" s="7"/>
@@ -6859,7 +6830,7 @@
       <c r="I295" s="7"/>
       <c r="K295" s="7"/>
       <c r="L295" s="7" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="M295" s="7"/>
@@ -6868,7 +6839,7 @@
     <row r="296">
       <c r="A296" s="6"/>
       <c r="B296" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="F296" s="7"/>
@@ -6876,7 +6847,7 @@
       <c r="I296" s="7"/>
       <c r="K296" s="7"/>
       <c r="L296" s="7" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="M296" s="7"/>
@@ -6885,7 +6856,7 @@
     <row r="297">
       <c r="A297" s="6"/>
       <c r="B297" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="F297" s="7"/>
@@ -6893,7 +6864,7 @@
       <c r="I297" s="7"/>
       <c r="K297" s="7"/>
       <c r="L297" s="7" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="M297" s="7"/>
@@ -6902,7 +6873,7 @@
     <row r="298">
       <c r="A298" s="6"/>
       <c r="B298" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="F298" s="7"/>
@@ -6910,7 +6881,7 @@
       <c r="I298" s="7"/>
       <c r="K298" s="7"/>
       <c r="L298" s="7" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="M298" s="7"/>
@@ -6919,7 +6890,7 @@
     <row r="299">
       <c r="A299" s="6"/>
       <c r="B299" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="F299" s="7"/>
@@ -6927,7 +6898,7 @@
       <c r="I299" s="7"/>
       <c r="K299" s="7"/>
       <c r="L299" s="7" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="M299" s="7"/>
@@ -6936,7 +6907,7 @@
     <row r="300">
       <c r="A300" s="6"/>
       <c r="B300" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="F300" s="7"/>
@@ -6944,7 +6915,7 @@
       <c r="I300" s="7"/>
       <c r="K300" s="7"/>
       <c r="L300" s="7" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="M300" s="7"/>
@@ -6953,7 +6924,7 @@
     <row r="301">
       <c r="A301" s="6"/>
       <c r="B301" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="F301" s="7"/>
@@ -6961,7 +6932,7 @@
       <c r="I301" s="7"/>
       <c r="K301" s="7"/>
       <c r="L301" s="7" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="M301" s="7"/>
@@ -6970,7 +6941,7 @@
     <row r="302">
       <c r="A302" s="6"/>
       <c r="B302" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="F302" s="7"/>
@@ -6978,7 +6949,7 @@
       <c r="I302" s="7"/>
       <c r="K302" s="7"/>
       <c r="L302" s="7" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="M302" s="7"/>
@@ -6987,7 +6958,7 @@
     <row r="303">
       <c r="A303" s="6"/>
       <c r="B303" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="F303" s="7"/>
@@ -6995,7 +6966,7 @@
       <c r="I303" s="7"/>
       <c r="K303" s="7"/>
       <c r="L303" s="7" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="M303" s="7"/>
@@ -7016,7 +6987,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="expression" priority="1" id="{2F66378E-610A-4AC9-BF2B-1C57091DB2EF}">
+          <x14:cfRule type="expression" priority="1" id="{AE8FE59E-AFE2-413D-AB4E-A4115AEFBA22}">
             <xm:f>N4="Completed"</xm:f>
             <x14:dxf>
               <font>
@@ -7033,7 +7004,7 @@
           <xm:sqref>N4:N303</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="expression" priority="2" id="{920D3AB1-1884-4B4C-9C1C-D072A2A2E175}">
+          <x14:cfRule type="expression" priority="2" id="{45438E3B-78A2-44A3-AC3F-D00227E909AC}">
             <xm:f>N4="Partial"</xm:f>
             <x14:dxf>
               <font>
@@ -7050,7 +7021,7 @@
           <xm:sqref>N4:N303</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="expression" priority="3" id="{97145B06-BE54-42C6-A58C-1305386F5540}">
+          <x14:cfRule type="expression" priority="3" id="{7CDAA07D-1945-462D-AAE7-54C2807A904B}">
             <xm:f>N4="Skipped"</xm:f>
             <x14:dxf>
               <font>
@@ -7070,19 +7041,19 @@
     </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="7" disablePrompts="0">
-        <x14:dataValidation xr:uid="{EADBC08C-A3E3-4460-B19D-6FB49909C4B7}" type="list" allowBlank="0" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+        <x14:dataValidation xr:uid="{3C066227-FAE6-4D6B-A481-B1B8FEE68F61}" type="list" allowBlank="0" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
           <x14:formula1>
             <xm:f>"Home Strength A,Home Strength B,Full-Body Gym,Rucking / Walking,Recovery,Other"</xm:f>
           </x14:formula1>
           <xm:sqref>C4 C7 C9 C11:C303 C6</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{BBAED253-40F9-442C-BC5F-0E22F0F7102F}" type="list" allowBlank="0" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+        <x14:dataValidation xr:uid="{B46A0D78-A8B9-403E-9839-CBF90E5B1A3E}" type="list" allowBlank="0" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
           <x14:formula1>
             <xm:f>"Completed,Partial,Skipped"</xm:f>
           </x14:formula1>
           <xm:sqref>N4:N5 N12:N303 N6 N7 N8 N9 N10 N11</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{1F793DC5-585C-45F6-A2F1-D123C28B7232}" type="decimal" allowBlank="0" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+        <x14:dataValidation xr:uid="{EF089D42-94FC-4A5A-AA25-A9CFF9F9A3EB}" type="decimal" allowBlank="0" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
           <x14:formula1>
             <xm:f>1</xm:f>
           </x14:formula1>
@@ -7091,19 +7062,19 @@
           </x14:formula2>
           <xm:sqref>K4 K8 K10:K303 K6</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{B1A865B4-4390-4946-B55E-D64D72625122}" type="list" allowBlank="0" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+        <x14:dataValidation xr:uid="{B1C6D477-FA71-4D17-A61D-3A65D8CF7F40}" type="list" allowBlank="0" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
           <x14:formula1>
             <xm:f>"Home Strength A,Home Strength B,Full-Body Gym,Rucking / Walking,Recovery,Other"</xm:f>
           </x14:formula1>
           <xm:sqref>C5</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{62960BF7-58C9-4FB7-B2B1-073B7A560E7F}" type="list" allowBlank="0" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+        <x14:dataValidation xr:uid="{26399F63-6959-4B6F-A207-50B543C0EE5E}" type="list" allowBlank="0" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
           <x14:formula1>
             <xm:f>"Home Strength A,Home Strength B,Full-Body Gym,Rucking / Walking,Recovery,Other"</xm:f>
           </x14:formula1>
           <xm:sqref>C8</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{AE98E89D-4334-48C2-B92F-1202FFC0DCB8}" type="decimal" allowBlank="0" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+        <x14:dataValidation xr:uid="{D75A90B2-1D59-4541-884D-C1291DECEBEF}" type="decimal" allowBlank="0" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
           <x14:formula1>
             <xm:f>1</xm:f>
           </x14:formula1>
@@ -7112,7 +7083,7 @@
           </x14:formula2>
           <xm:sqref>K7</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{E939CA86-E07A-47C5-AF2A-E82A877E4016}" type="list" allowBlank="0" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+        <x14:dataValidation xr:uid="{140282BF-0910-4B10-8828-930FF200FA61}" type="list" allowBlank="0" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
           <x14:formula1>
             <xm:f>"Home Strength A,Home Strength B,Full-Body Gym,Rucking / Walking,Recovery,Other"</xm:f>
           </x14:formula1>

</xml_diff>